<commit_message>
feat(modules): migrar páginas configuracion, vehiculos, vendedores a módulos
- Agregadas funciones faltantes al módulo vendedores: getVendedoresStats, VendedorStats, createMultipleVendedores
- Configuración: importa de @/modules/configuracion
- Vehículos: importa de @/modules/vehiculos
- Vendedores: importa de @/modules/vendedores
</commit_message>
<xml_diff>
--- a/Vehiculos/Vehiculos FULL.xlsx
+++ b/Vehiculos/Vehiculos FULL.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Vehiculos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AI\Antigravity\FALPAT Ventas\Vehiculos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C74A8A21-F2BF-4827-952A-CDA897FF6735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1080" windowWidth="14280" windowHeight="9720" xr2:uid="{EEE76CC5-F6C5-4087-9D34-9E33F1DCF93B}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4485"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -18,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$K$31</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="153">
   <si>
     <t>Patente</t>
   </si>
@@ -484,12 +483,27 @@
   </si>
   <si>
     <t>M-3529</t>
+  </si>
+  <si>
+    <t>NYR481</t>
+  </si>
+  <si>
+    <t>Iveco</t>
+  </si>
+  <si>
+    <t>TRAKKER 410</t>
+  </si>
+  <si>
+    <t>WJMJ3JJSS40C193012</t>
+  </si>
+  <si>
+    <t>R069099623</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -834,24 +848,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E8134D6-A8A1-4E25-8C8E-CDB120757F44}">
-  <dimension ref="A1:K31"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.90625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.36328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.7265625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="31.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="31.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -886,7 +900,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>141</v>
       </c>
@@ -921,7 +935,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>110</v>
       </c>
@@ -956,7 +970,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>34</v>
       </c>
@@ -991,7 +1005,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -1026,7 +1040,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>72</v>
       </c>
@@ -1061,7 +1075,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>30</v>
       </c>
@@ -1096,7 +1110,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>68</v>
       </c>
@@ -1131,7 +1145,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>64</v>
       </c>
@@ -1166,7 +1180,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>81</v>
       </c>
@@ -1201,7 +1215,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>77</v>
       </c>
@@ -1236,7 +1250,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>107</v>
       </c>
@@ -1271,7 +1285,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -1306,7 +1320,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>145</v>
       </c>
@@ -1341,7 +1355,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>117</v>
       </c>
@@ -1376,7 +1390,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>101</v>
       </c>
@@ -1411,7 +1425,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>126</v>
       </c>
@@ -1446,7 +1460,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>131</v>
       </c>
@@ -1481,7 +1495,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>58</v>
       </c>
@@ -1516,7 +1530,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>89</v>
       </c>
@@ -1551,7 +1565,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>37</v>
       </c>
@@ -1586,7 +1600,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>44</v>
       </c>
@@ -1621,7 +1635,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>98</v>
       </c>
@@ -1656,7 +1670,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>94</v>
       </c>
@@ -1691,7 +1705,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>85</v>
       </c>
@@ -1726,7 +1740,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>48</v>
       </c>
@@ -1761,7 +1775,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>113</v>
       </c>
@@ -1796,7 +1810,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>55</v>
       </c>
@@ -1831,7 +1845,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>11</v>
       </c>
@@ -1866,7 +1880,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>136</v>
       </c>
@@ -1901,7 +1915,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>121</v>
       </c>
@@ -1936,7 +1950,43 @@
         <v>29</v>
       </c>
     </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>148</v>
+      </c>
+      <c r="B32" t="s">
+        <v>149</v>
+      </c>
+      <c r="C32" t="s">
+        <v>150</v>
+      </c>
+      <c r="D32">
+        <v>2014</v>
+      </c>
+      <c r="E32" t="s">
+        <v>151</v>
+      </c>
+      <c r="F32" t="s">
+        <v>152</v>
+      </c>
+      <c r="G32" t="s">
+        <v>18</v>
+      </c>
+      <c r="H32" t="s">
+        <v>18</v>
+      </c>
+      <c r="I32" t="s">
+        <v>18</v>
+      </c>
+      <c r="J32" t="s">
+        <v>18</v>
+      </c>
+      <c r="K32" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:K31"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Deploy: add render.yaml, 5 tareas completadas
- Backup script actualizado (exporta todas las colecciones)
- Entregas carga remitos_aprobados
- Paginacion UI (20 items/pagina) en Presupuestos, Remitos, Facturacion
- Dashboard usa getCountFromServer para clientes
- UI: 'Entrega' -> 'Salida', 'A Entregar' -> 'A Despachar'
- Fix hydration error (button anidados -> divs)
- render.yaml para Render deploy
</commit_message>
<xml_diff>
--- a/Vehiculos/Vehiculos FULL.xlsx
+++ b/Vehiculos/Vehiculos FULL.xlsx
@@ -513,12 +513,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -533,8 +539,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1950,38 +1957,38 @@
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row r="32" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="D32">
+      <c r="D32" s="1">
         <v>2014</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E32" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F32" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="G32" t="s">
-        <v>18</v>
-      </c>
-      <c r="H32" t="s">
-        <v>18</v>
-      </c>
-      <c r="I32" t="s">
-        <v>18</v>
-      </c>
-      <c r="J32" t="s">
-        <v>18</v>
-      </c>
-      <c r="K32" t="s">
+      <c r="G32" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K32" s="1" t="s">
         <v>33</v>
       </c>
     </row>

</xml_diff>